<commit_message>
Counting how many sites in the RLS mind map
</commit_message>
<xml_diff>
--- a/RLS_Sampling.xlsx
+++ b/RLS_Sampling.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecjones/Documents/GitHub/Alec_Jones_Honours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F63859C4-3356-A148-A3D4-F68855A33BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEDC907E-EC7F-534E-BDD3-B0FC5AF85268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="500" windowWidth="28800" windowHeight="16040" xr2:uid="{2EAAD8B1-2ED3-8949-A54D-067544EBCB23}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16040" xr2:uid="{2EAAD8B1-2ED3-8949-A54D-067544EBCB23}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL_BY_YEAR" sheetId="1" r:id="rId1"/>
@@ -1521,71 +1521,71 @@
     <xf numFmtId="49" fontId="4" fillId="17" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2001,42 +2001,42 @@
       <c r="O1" s="131"/>
       <c r="P1" s="131"/>
       <c r="Q1" s="131"/>
-      <c r="R1" s="125" t="s">
+      <c r="R1" s="124" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="126"/>
-      <c r="T1" s="126"/>
-      <c r="U1" s="126"/>
-      <c r="V1" s="126"/>
-      <c r="W1" s="127"/>
-      <c r="X1" s="124" t="s">
+      <c r="S1" s="125"/>
+      <c r="T1" s="125"/>
+      <c r="U1" s="125"/>
+      <c r="V1" s="125"/>
+      <c r="W1" s="126"/>
+      <c r="X1" s="123" t="s">
         <v>48</v>
       </c>
-      <c r="Y1" s="124"/>
-      <c r="Z1" s="124"/>
-      <c r="AA1" s="124"/>
-      <c r="AB1" s="124"/>
-      <c r="AC1" s="124"/>
+      <c r="Y1" s="123"/>
+      <c r="Z1" s="123"/>
+      <c r="AA1" s="123"/>
+      <c r="AB1" s="123"/>
+      <c r="AC1" s="123"/>
       <c r="AD1" s="128" t="s">
         <v>63</v>
       </c>
-      <c r="AE1" s="124"/>
-      <c r="AF1" s="124"/>
-      <c r="AG1" s="124"/>
-      <c r="AH1" s="124"/>
+      <c r="AE1" s="123"/>
+      <c r="AF1" s="123"/>
+      <c r="AG1" s="123"/>
+      <c r="AH1" s="123"/>
       <c r="AI1" s="129"/>
-      <c r="AJ1" s="122" t="s">
+      <c r="AJ1" s="121" t="s">
         <v>66</v>
       </c>
-      <c r="AK1" s="122"/>
-      <c r="AL1" s="122"/>
-      <c r="AM1" s="122"/>
-      <c r="AN1" s="122"/>
-      <c r="AO1" s="122"/>
-      <c r="AP1" s="123"/>
+      <c r="AK1" s="121"/>
+      <c r="AL1" s="121"/>
+      <c r="AM1" s="121"/>
+      <c r="AN1" s="121"/>
+      <c r="AO1" s="121"/>
+      <c r="AP1" s="122"/>
     </row>
     <row r="2" spans="1:42" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="116" t="s">
+      <c r="A2" s="127" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -2135,7 +2135,7 @@
       <c r="AP2" s="39"/>
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A3" s="116"/>
+      <c r="A3" s="127"/>
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
@@ -2243,7 +2243,7 @@
       <c r="AP3" s="8"/>
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A4" s="116"/>
+      <c r="A4" s="127"/>
       <c r="B4" s="1" t="s">
         <v>42</v>
       </c>
@@ -2297,11 +2297,11 @@
       <c r="AP4" s="8"/>
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A5" s="116"/>
-      <c r="B5" s="118" t="s">
+      <c r="A5" s="127"/>
+      <c r="B5" s="119" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="118" t="s">
+      <c r="C5" s="119" t="s">
         <v>34</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -2347,9 +2347,9 @@
       <c r="AP5" s="8"/>
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A6" s="116"/>
-      <c r="B6" s="118"/>
-      <c r="C6" s="118"/>
+      <c r="A6" s="127"/>
+      <c r="B6" s="119"/>
+      <c r="C6" s="119"/>
       <c r="D6" s="3" t="s">
         <v>18</v>
       </c>
@@ -2455,7 +2455,7 @@
       <c r="AP6" s="8"/>
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A7" s="116"/>
+      <c r="A7" s="127"/>
       <c r="B7" s="3" t="s">
         <v>43</v>
       </c>
@@ -2510,7 +2510,7 @@
       <c r="AP7" s="8"/>
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A8" s="116"/>
+      <c r="A8" s="127"/>
       <c r="B8" s="3" t="s">
         <v>44</v>
       </c>
@@ -2566,7 +2566,7 @@
       <c r="AP8" s="10"/>
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A9" s="116"/>
+      <c r="A9" s="127"/>
       <c r="B9" s="3" t="s">
         <v>45</v>
       </c>
@@ -2622,7 +2622,7 @@
       <c r="AP9" s="10"/>
     </row>
     <row r="10" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A10" s="116"/>
+      <c r="A10" s="127"/>
       <c r="B10" s="3" t="s">
         <v>46</v>
       </c>
@@ -2678,7 +2678,7 @@
       <c r="AP10" s="10"/>
     </row>
     <row r="11" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A11" s="116"/>
+      <c r="A11" s="127"/>
       <c r="B11" s="3" t="s">
         <v>47</v>
       </c>
@@ -2734,11 +2734,11 @@
       <c r="AP11" s="10"/>
     </row>
     <row r="12" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A12" s="116"/>
-      <c r="B12" s="118" t="s">
+      <c r="A12" s="127"/>
+      <c r="B12" s="119" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="118" t="s">
+      <c r="C12" s="119" t="s">
         <v>22</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -2790,9 +2790,9 @@
       <c r="AP12" s="10"/>
     </row>
     <row r="13" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A13" s="116"/>
-      <c r="B13" s="118"/>
-      <c r="C13" s="118"/>
+      <c r="A13" s="127"/>
+      <c r="B13" s="119"/>
+      <c r="C13" s="119"/>
       <c r="D13" s="1" t="s">
         <v>24</v>
       </c>
@@ -2841,9 +2841,9 @@
       <c r="AP13" s="10"/>
     </row>
     <row r="14" spans="1:42" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="116"/>
-      <c r="B14" s="118"/>
-      <c r="C14" s="118"/>
+      <c r="A14" s="127"/>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
       <c r="D14" s="1" t="s">
         <v>18</v>
       </c>
@@ -2892,7 +2892,7 @@
       <c r="AP14" s="10"/>
     </row>
     <row r="15" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A15" s="116"/>
+      <c r="A15" s="127"/>
       <c r="B15" s="3" t="s">
         <v>39</v>
       </c>
@@ -2948,11 +2948,11 @@
       <c r="AP15" s="10"/>
     </row>
     <row r="16" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A16" s="116"/>
-      <c r="B16" s="118" t="s">
+      <c r="A16" s="127"/>
+      <c r="B16" s="119" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="118" t="s">
+      <c r="C16" s="119" t="s">
         <v>20</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -3004,9 +3004,9 @@
       <c r="AP16" s="10"/>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A17" s="116"/>
-      <c r="B17" s="118"/>
-      <c r="C17" s="118"/>
+      <c r="A17" s="127"/>
+      <c r="B17" s="119"/>
+      <c r="C17" s="119"/>
       <c r="D17" s="1" t="s">
         <v>17</v>
       </c>
@@ -3055,9 +3055,9 @@
       <c r="AP17" s="10"/>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A18" s="116"/>
-      <c r="B18" s="118"/>
-      <c r="C18" s="118"/>
+      <c r="A18" s="127"/>
+      <c r="B18" s="119"/>
+      <c r="C18" s="119"/>
       <c r="D18" s="1" t="s">
         <v>18</v>
       </c>
@@ -3115,11 +3115,11 @@
       <c r="AP18" s="10"/>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A19" s="116"/>
-      <c r="B19" s="118" t="s">
+      <c r="A19" s="127"/>
+      <c r="B19" s="119" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="118" t="s">
+      <c r="C19" s="119" t="s">
         <v>36</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -3169,9 +3169,9 @@
       <c r="AP19" s="10"/>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A20" s="116"/>
-      <c r="B20" s="118"/>
-      <c r="C20" s="118"/>
+      <c r="A20" s="127"/>
+      <c r="B20" s="119"/>
+      <c r="C20" s="119"/>
       <c r="D20" s="1" t="s">
         <v>24</v>
       </c>
@@ -3215,9 +3215,9 @@
       <c r="AP20" s="10"/>
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A21" s="116"/>
-      <c r="B21" s="118"/>
-      <c r="C21" s="118"/>
+      <c r="A21" s="127"/>
+      <c r="B21" s="119"/>
+      <c r="C21" s="119"/>
       <c r="D21" s="1" t="s">
         <v>18</v>
       </c>
@@ -3296,7 +3296,7 @@
       <c r="AP21" s="10"/>
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A22" s="116"/>
+      <c r="A22" s="127"/>
       <c r="B22" s="3" t="s">
         <v>4</v>
       </c>
@@ -3351,7 +3351,7 @@
       <c r="AP22" s="10"/>
     </row>
     <row r="23" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A23" s="116"/>
+      <c r="A23" s="127"/>
       <c r="B23" s="3" t="s">
         <v>7</v>
       </c>
@@ -3406,7 +3406,7 @@
       <c r="AP23" s="10"/>
     </row>
     <row r="24" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A24" s="116"/>
+      <c r="A24" s="127"/>
       <c r="B24" s="3" t="s">
         <v>9</v>
       </c>
@@ -3463,7 +3463,7 @@
       <c r="AP24" s="10"/>
     </row>
     <row r="25" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A25" s="116"/>
+      <c r="A25" s="127"/>
       <c r="B25" s="3" t="s">
         <v>25</v>
       </c>
@@ -3518,7 +3518,7 @@
       <c r="AP25" s="10"/>
     </row>
     <row r="26" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A26" s="116"/>
+      <c r="A26" s="127"/>
       <c r="B26" s="3" t="s">
         <v>25</v>
       </c>
@@ -3573,11 +3573,11 @@
       <c r="AP26" s="10"/>
     </row>
     <row r="27" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A27" s="116"/>
-      <c r="B27" s="118" t="s">
+      <c r="A27" s="127"/>
+      <c r="B27" s="119" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="118" t="s">
+      <c r="C27" s="119" t="s">
         <v>27</v>
       </c>
       <c r="D27" s="3" t="s">
@@ -3628,9 +3628,9 @@
       <c r="AP27" s="10"/>
     </row>
     <row r="28" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A28" s="116"/>
-      <c r="B28" s="118"/>
-      <c r="C28" s="118"/>
+      <c r="A28" s="127"/>
+      <c r="B28" s="119"/>
+      <c r="C28" s="119"/>
       <c r="D28" s="3" t="s">
         <v>17</v>
       </c>
@@ -3679,7 +3679,7 @@
       <c r="AP28" s="10"/>
     </row>
     <row r="29" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A29" s="116"/>
+      <c r="A29" s="127"/>
       <c r="B29" s="3" t="s">
         <v>30</v>
       </c>
@@ -3736,7 +3736,7 @@
       <c r="AP29" s="10"/>
     </row>
     <row r="30" spans="1:43" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="116"/>
+      <c r="A30" s="127"/>
       <c r="B30" s="3" t="s">
         <v>37</v>
       </c>
@@ -3800,13 +3800,13 @@
       <c r="AP30" s="10"/>
     </row>
     <row r="31" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A31" s="115" t="s">
+      <c r="A31" s="133" t="s">
         <v>89</v>
       </c>
-      <c r="B31" s="134" t="s">
+      <c r="B31" s="117" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="134" t="s">
+      <c r="C31" s="117" t="s">
         <v>90</v>
       </c>
       <c r="D31" s="40" t="s">
@@ -3893,9 +3893,9 @@
       </c>
     </row>
     <row r="32" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A32" s="116"/>
-      <c r="B32" s="121"/>
-      <c r="C32" s="121"/>
+      <c r="A32" s="127"/>
+      <c r="B32" s="118"/>
+      <c r="C32" s="118"/>
       <c r="D32" s="1" t="s">
         <v>18</v>
       </c>
@@ -3955,7 +3955,7 @@
       </c>
     </row>
     <row r="33" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A33" s="116"/>
+      <c r="A33" s="127"/>
       <c r="B33" s="1" t="s">
         <v>68</v>
       </c>
@@ -4030,7 +4030,7 @@
       </c>
     </row>
     <row r="34" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A34" s="116"/>
+      <c r="A34" s="127"/>
       <c r="B34" s="1" t="s">
         <v>69</v>
       </c>
@@ -4114,7 +4114,7 @@
       </c>
     </row>
     <row r="35" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A35" s="116"/>
+      <c r="A35" s="127"/>
       <c r="B35" s="1" t="s">
         <v>70</v>
       </c>
@@ -4189,11 +4189,11 @@
       </c>
     </row>
     <row r="36" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A36" s="116"/>
-      <c r="B36" s="121" t="s">
+      <c r="A36" s="127"/>
+      <c r="B36" s="118" t="s">
         <v>71</v>
       </c>
-      <c r="C36" s="121" t="s">
+      <c r="C36" s="118" t="s">
         <v>97</v>
       </c>
       <c r="D36" s="1" t="s">
@@ -4273,9 +4273,9 @@
       </c>
     </row>
     <row r="37" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A37" s="116"/>
-      <c r="B37" s="121"/>
-      <c r="C37" s="121"/>
+      <c r="A37" s="127"/>
+      <c r="B37" s="118"/>
+      <c r="C37" s="118"/>
       <c r="D37" s="1" t="s">
         <v>29</v>
       </c>
@@ -4342,7 +4342,7 @@
       </c>
     </row>
     <row r="38" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A38" s="116"/>
+      <c r="A38" s="127"/>
       <c r="B38" s="1" t="s">
         <v>72</v>
       </c>
@@ -4433,7 +4433,7 @@
       </c>
     </row>
     <row r="39" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A39" s="116"/>
+      <c r="A39" s="127"/>
       <c r="B39" s="1" t="s">
         <v>73</v>
       </c>
@@ -4492,11 +4492,11 @@
       </c>
     </row>
     <row r="40" spans="1:43" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="116"/>
-      <c r="B40" s="133" t="s">
+      <c r="A40" s="127"/>
+      <c r="B40" s="120" t="s">
         <v>74</v>
       </c>
-      <c r="C40" s="118" t="s">
+      <c r="C40" s="119" t="s">
         <v>100</v>
       </c>
       <c r="D40" s="1" t="s">
@@ -4556,9 +4556,9 @@
       </c>
     </row>
     <row r="41" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A41" s="116"/>
-      <c r="B41" s="133"/>
-      <c r="C41" s="118"/>
+      <c r="A41" s="127"/>
+      <c r="B41" s="120"/>
+      <c r="C41" s="119"/>
       <c r="D41" s="1" t="s">
         <v>29</v>
       </c>
@@ -4638,7 +4638,7 @@
       </c>
     </row>
     <row r="42" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A42" s="116"/>
+      <c r="A42" s="127"/>
       <c r="B42" s="1" t="s">
         <v>75</v>
       </c>
@@ -4724,11 +4724,11 @@
       </c>
     </row>
     <row r="43" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A43" s="116"/>
-      <c r="B43" s="121" t="s">
+      <c r="A43" s="127"/>
+      <c r="B43" s="118" t="s">
         <v>76</v>
       </c>
-      <c r="C43" s="118" t="s">
+      <c r="C43" s="119" t="s">
         <v>121</v>
       </c>
       <c r="D43" s="1" t="s">
@@ -4786,9 +4786,9 @@
       </c>
     </row>
     <row r="44" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A44" s="116"/>
-      <c r="B44" s="121"/>
-      <c r="C44" s="118"/>
+      <c r="A44" s="127"/>
+      <c r="B44" s="118"/>
+      <c r="C44" s="119"/>
       <c r="D44" s="1" t="s">
         <v>94</v>
       </c>
@@ -4868,7 +4868,7 @@
       </c>
     </row>
     <row r="45" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A45" s="116"/>
+      <c r="A45" s="127"/>
       <c r="B45" s="1" t="s">
         <v>77</v>
       </c>
@@ -4959,11 +4959,11 @@
       </c>
     </row>
     <row r="46" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A46" s="116"/>
-      <c r="B46" s="121" t="s">
+      <c r="A46" s="127"/>
+      <c r="B46" s="118" t="s">
         <v>78</v>
       </c>
-      <c r="C46" s="118" t="s">
+      <c r="C46" s="119" t="s">
         <v>103</v>
       </c>
       <c r="D46" s="1" t="s">
@@ -5024,9 +5024,9 @@
       </c>
     </row>
     <row r="47" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A47" s="116"/>
-      <c r="B47" s="121"/>
-      <c r="C47" s="118"/>
+      <c r="A47" s="127"/>
+      <c r="B47" s="118"/>
+      <c r="C47" s="119"/>
       <c r="D47" s="1" t="s">
         <v>17</v>
       </c>
@@ -5106,7 +5106,7 @@
       </c>
     </row>
     <row r="48" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A48" s="116"/>
+      <c r="A48" s="127"/>
       <c r="B48" s="1" t="s">
         <v>79</v>
       </c>
@@ -5176,7 +5176,7 @@
       </c>
     </row>
     <row r="49" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A49" s="116"/>
+      <c r="A49" s="127"/>
       <c r="B49" s="1" t="s">
         <v>80</v>
       </c>
@@ -5246,7 +5246,7 @@
       </c>
     </row>
     <row r="50" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A50" s="116"/>
+      <c r="A50" s="127"/>
       <c r="B50" s="1" t="s">
         <v>81</v>
       </c>
@@ -5316,7 +5316,7 @@
       </c>
     </row>
     <row r="51" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A51" s="116"/>
+      <c r="A51" s="127"/>
       <c r="B51" s="1" t="s">
         <v>82</v>
       </c>
@@ -5386,7 +5386,7 @@
       </c>
     </row>
     <row r="52" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A52" s="116"/>
+      <c r="A52" s="127"/>
       <c r="B52" s="1" t="s">
         <v>83</v>
       </c>
@@ -5456,7 +5456,7 @@
       </c>
     </row>
     <row r="53" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A53" s="116"/>
+      <c r="A53" s="127"/>
       <c r="B53" s="1" t="s">
         <v>84</v>
       </c>
@@ -5526,7 +5526,7 @@
       </c>
     </row>
     <row r="54" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A54" s="116"/>
+      <c r="A54" s="127"/>
       <c r="B54" s="1" t="s">
         <v>85</v>
       </c>
@@ -5612,7 +5612,7 @@
       </c>
     </row>
     <row r="55" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A55" s="116"/>
+      <c r="A55" s="127"/>
       <c r="B55" s="1" t="s">
         <v>86</v>
       </c>
@@ -5698,7 +5698,7 @@
       </c>
     </row>
     <row r="56" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A56" s="116"/>
+      <c r="A56" s="127"/>
       <c r="B56" s="1" t="s">
         <v>87</v>
       </c>
@@ -5784,7 +5784,7 @@
       </c>
     </row>
     <row r="57" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A57" s="116"/>
+      <c r="A57" s="127"/>
       <c r="B57" s="1" t="s">
         <v>88</v>
       </c>
@@ -5870,7 +5870,7 @@
       </c>
     </row>
     <row r="58" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A58" s="116"/>
+      <c r="A58" s="127"/>
       <c r="B58" s="1" t="s">
         <v>117</v>
       </c>
@@ -5942,11 +5942,11 @@
       </c>
     </row>
     <row r="59" spans="1:43" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="116"/>
-      <c r="B59" s="121" t="s">
+      <c r="A59" s="127"/>
+      <c r="B59" s="118" t="s">
         <v>123</v>
       </c>
-      <c r="C59" s="121" t="s">
+      <c r="C59" s="118" t="s">
         <v>127</v>
       </c>
       <c r="D59" s="1" t="s">
@@ -6001,9 +6001,9 @@
       </c>
     </row>
     <row r="60" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A60" s="116"/>
-      <c r="B60" s="121"/>
-      <c r="C60" s="121"/>
+      <c r="A60" s="127"/>
+      <c r="B60" s="118"/>
+      <c r="C60" s="118"/>
       <c r="D60" s="1" t="s">
         <v>17</v>
       </c>
@@ -6061,11 +6061,11 @@
       </c>
     </row>
     <row r="61" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A61" s="116"/>
-      <c r="B61" s="121" t="s">
+      <c r="A61" s="127"/>
+      <c r="B61" s="118" t="s">
         <v>124</v>
       </c>
-      <c r="C61" s="118" t="s">
+      <c r="C61" s="119" t="s">
         <v>128</v>
       </c>
       <c r="D61" s="1" t="s">
@@ -6125,9 +6125,9 @@
       </c>
     </row>
     <row r="62" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A62" s="116"/>
-      <c r="B62" s="121"/>
-      <c r="C62" s="118"/>
+      <c r="A62" s="127"/>
+      <c r="B62" s="118"/>
+      <c r="C62" s="119"/>
       <c r="D62" s="1" t="s">
         <v>129</v>
       </c>
@@ -6185,11 +6185,11 @@
       </c>
     </row>
     <row r="63" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A63" s="116"/>
-      <c r="B63" s="121" t="s">
+      <c r="A63" s="127"/>
+      <c r="B63" s="118" t="s">
         <v>125</v>
       </c>
-      <c r="C63" s="118" t="s">
+      <c r="C63" s="119" t="s">
         <v>131</v>
       </c>
       <c r="D63" s="1" t="s">
@@ -6249,9 +6249,9 @@
       </c>
     </row>
     <row r="64" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A64" s="116"/>
-      <c r="B64" s="121"/>
-      <c r="C64" s="118"/>
+      <c r="A64" s="127"/>
+      <c r="B64" s="118"/>
+      <c r="C64" s="119"/>
       <c r="D64" s="1" t="s">
         <v>18</v>
       </c>
@@ -6309,7 +6309,7 @@
       </c>
     </row>
     <row r="65" spans="1:43" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="116"/>
+      <c r="A65" s="127"/>
       <c r="B65" s="1" t="s">
         <v>126</v>
       </c>
@@ -6378,7 +6378,7 @@
       </c>
     </row>
     <row r="66" spans="1:43" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="115" t="s">
+      <c r="A66" s="133" t="s">
         <v>140</v>
       </c>
       <c r="B66" s="40" t="s">
@@ -6444,11 +6444,11 @@
       <c r="AP66" s="39"/>
     </row>
     <row r="67" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A67" s="116"/>
-      <c r="B67" s="121" t="s">
+      <c r="A67" s="127"/>
+      <c r="B67" s="118" t="s">
         <v>152</v>
       </c>
-      <c r="C67" s="121" t="s">
+      <c r="C67" s="118" t="s">
         <v>153</v>
       </c>
       <c r="D67" s="1" t="s">
@@ -6505,9 +6505,9 @@
       <c r="AP67" s="8"/>
     </row>
     <row r="68" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A68" s="116"/>
-      <c r="B68" s="121"/>
-      <c r="C68" s="121"/>
+      <c r="A68" s="127"/>
+      <c r="B68" s="118"/>
+      <c r="C68" s="118"/>
       <c r="D68" s="1" t="s">
         <v>18</v>
       </c>
@@ -6562,11 +6562,11 @@
       <c r="AP68" s="8"/>
     </row>
     <row r="69" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A69" s="116"/>
-      <c r="B69" s="121" t="s">
+      <c r="A69" s="127"/>
+      <c r="B69" s="118" t="s">
         <v>154</v>
       </c>
-      <c r="C69" s="121" t="s">
+      <c r="C69" s="118" t="s">
         <v>155</v>
       </c>
       <c r="D69" s="1" t="s">
@@ -6623,9 +6623,9 @@
       <c r="AP69" s="8"/>
     </row>
     <row r="70" spans="1:43" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="117"/>
-      <c r="B70" s="121"/>
-      <c r="C70" s="121"/>
+      <c r="A70" s="134"/>
+      <c r="B70" s="118"/>
+      <c r="C70" s="118"/>
       <c r="D70" s="1" t="s">
         <v>29</v>
       </c>
@@ -6681,7 +6681,7 @@
       <c r="AP70" s="47"/>
     </row>
     <row r="71" spans="1:43" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="119" t="s">
+      <c r="A71" s="135" t="s">
         <v>141</v>
       </c>
       <c r="B71" s="40" t="s">
@@ -6744,7 +6744,7 @@
       <c r="AP71" s="8"/>
     </row>
     <row r="72" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A72" s="120"/>
+      <c r="A72" s="136"/>
       <c r="B72" s="1" t="s">
         <v>146</v>
       </c>
@@ -6805,7 +6805,7 @@
       <c r="AP72" s="8"/>
     </row>
     <row r="73" spans="1:43" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="120"/>
+      <c r="A73" s="136"/>
       <c r="B73" s="1" t="s">
         <v>148</v>
       </c>
@@ -6866,13 +6866,13 @@
       <c r="AP73" s="8"/>
     </row>
     <row r="74" spans="1:43" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="115" t="s">
+      <c r="A74" s="133" t="s">
         <v>143</v>
       </c>
-      <c r="B74" s="134" t="s">
+      <c r="B74" s="117" t="s">
         <v>157</v>
       </c>
-      <c r="C74" s="135" t="s">
+      <c r="C74" s="115" t="s">
         <v>165</v>
       </c>
       <c r="D74" s="40" t="s">
@@ -6930,9 +6930,9 @@
       <c r="AP74" s="39"/>
     </row>
     <row r="75" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A75" s="116"/>
-      <c r="B75" s="121"/>
-      <c r="C75" s="136"/>
+      <c r="A75" s="127"/>
+      <c r="B75" s="118"/>
+      <c r="C75" s="116"/>
       <c r="D75" s="1" t="s">
         <v>17</v>
       </c>
@@ -6987,7 +6987,7 @@
       <c r="AP75" s="8"/>
     </row>
     <row r="76" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A76" s="116"/>
+      <c r="A76" s="127"/>
       <c r="B76" s="3" t="s">
         <v>171</v>
       </c>
@@ -7050,7 +7050,7 @@
       </c>
     </row>
     <row r="77" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A77" s="116"/>
+      <c r="A77" s="127"/>
       <c r="B77" s="3" t="s">
         <v>172</v>
       </c>
@@ -7114,11 +7114,11 @@
       <c r="AP77" s="8"/>
     </row>
     <row r="78" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A78" s="116"/>
-      <c r="B78" s="118" t="s">
+      <c r="A78" s="127"/>
+      <c r="B78" s="119" t="s">
         <v>173</v>
       </c>
-      <c r="C78" s="118" t="s">
+      <c r="C78" s="119" t="s">
         <v>169</v>
       </c>
       <c r="D78" s="1" t="s">
@@ -7175,9 +7175,9 @@
       <c r="AP78" s="8"/>
     </row>
     <row r="79" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A79" s="116"/>
-      <c r="B79" s="118"/>
-      <c r="C79" s="118"/>
+      <c r="A79" s="127"/>
+      <c r="B79" s="119"/>
+      <c r="C79" s="119"/>
       <c r="D79" s="1" t="s">
         <v>94</v>
       </c>
@@ -7232,7 +7232,7 @@
       <c r="AP79" s="8"/>
     </row>
     <row r="80" spans="1:43" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="117"/>
+      <c r="A80" s="134"/>
       <c r="B80" s="99" t="s">
         <v>174</v>
       </c>
@@ -7335,35 +7335,6 @@
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="C74:C75"/>
-    <mergeCell ref="B74:B75"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="C63:C64"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="AJ1:AP1"/>
-    <mergeCell ref="X1:AC1"/>
-    <mergeCell ref="R1:W1"/>
-    <mergeCell ref="A2:A30"/>
-    <mergeCell ref="AD1:AI1"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="F1:K1"/>
-    <mergeCell ref="L1:Q1"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
     <mergeCell ref="A74:A80"/>
     <mergeCell ref="B12:B14"/>
     <mergeCell ref="C12:C14"/>
@@ -7380,6 +7351,35 @@
     <mergeCell ref="A31:A65"/>
     <mergeCell ref="B43:B44"/>
     <mergeCell ref="C43:C44"/>
+    <mergeCell ref="AJ1:AP1"/>
+    <mergeCell ref="X1:AC1"/>
+    <mergeCell ref="R1:W1"/>
+    <mergeCell ref="A2:A30"/>
+    <mergeCell ref="AD1:AI1"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="L1:Q1"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="C74:C75"/>
+    <mergeCell ref="B74:B75"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="C63:C64"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="E1:E1048576">

</xml_diff>

<commit_message>
Adding the rest of the data files from RLS
</commit_message>
<xml_diff>
--- a/RLS_Sampling.xlsx
+++ b/RLS_Sampling.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecjones/Documents/GitHub/Alec_Jones_Honours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEDC907E-EC7F-534E-BDD3-B0FC5AF85268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A91201-E5D3-1446-B14D-631906902248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16040" xr2:uid="{2EAAD8B1-2ED3-8949-A54D-067544EBCB23}"/>
+    <workbookView xWindow="-28800" yWindow="4100" windowWidth="28800" windowHeight="16040" xr2:uid="{2EAAD8B1-2ED3-8949-A54D-067544EBCB23}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL_BY_YEAR" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Finding dates from the surveys
</commit_message>
<xml_diff>
--- a/RLS_Sampling.xlsx
+++ b/RLS_Sampling.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecjones/Documents/GitHub/Alec_Jones_Honours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A91201-E5D3-1446-B14D-631906902248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32609811-2E1E-7C4A-A911-BBB0CFC42B7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="4100" windowWidth="28800" windowHeight="16040" xr2:uid="{2EAAD8B1-2ED3-8949-A54D-067544EBCB23}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" xr2:uid="{2EAAD8B1-2ED3-8949-A54D-067544EBCB23}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL_BY_YEAR" sheetId="1" r:id="rId1"/>
@@ -1521,71 +1521,71 @@
     <xf numFmtId="49" fontId="4" fillId="17" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2001,42 +2001,42 @@
       <c r="O1" s="131"/>
       <c r="P1" s="131"/>
       <c r="Q1" s="131"/>
-      <c r="R1" s="124" t="s">
+      <c r="R1" s="125" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="125"/>
-      <c r="T1" s="125"/>
-      <c r="U1" s="125"/>
-      <c r="V1" s="125"/>
-      <c r="W1" s="126"/>
-      <c r="X1" s="123" t="s">
+      <c r="S1" s="126"/>
+      <c r="T1" s="126"/>
+      <c r="U1" s="126"/>
+      <c r="V1" s="126"/>
+      <c r="W1" s="127"/>
+      <c r="X1" s="124" t="s">
         <v>48</v>
       </c>
-      <c r="Y1" s="123"/>
-      <c r="Z1" s="123"/>
-      <c r="AA1" s="123"/>
-      <c r="AB1" s="123"/>
-      <c r="AC1" s="123"/>
+      <c r="Y1" s="124"/>
+      <c r="Z1" s="124"/>
+      <c r="AA1" s="124"/>
+      <c r="AB1" s="124"/>
+      <c r="AC1" s="124"/>
       <c r="AD1" s="128" t="s">
         <v>63</v>
       </c>
-      <c r="AE1" s="123"/>
-      <c r="AF1" s="123"/>
-      <c r="AG1" s="123"/>
-      <c r="AH1" s="123"/>
+      <c r="AE1" s="124"/>
+      <c r="AF1" s="124"/>
+      <c r="AG1" s="124"/>
+      <c r="AH1" s="124"/>
       <c r="AI1" s="129"/>
-      <c r="AJ1" s="121" t="s">
+      <c r="AJ1" s="122" t="s">
         <v>66</v>
       </c>
-      <c r="AK1" s="121"/>
-      <c r="AL1" s="121"/>
-      <c r="AM1" s="121"/>
-      <c r="AN1" s="121"/>
-      <c r="AO1" s="121"/>
-      <c r="AP1" s="122"/>
+      <c r="AK1" s="122"/>
+      <c r="AL1" s="122"/>
+      <c r="AM1" s="122"/>
+      <c r="AN1" s="122"/>
+      <c r="AO1" s="122"/>
+      <c r="AP1" s="123"/>
     </row>
     <row r="2" spans="1:42" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="127" t="s">
+      <c r="A2" s="116" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -2135,7 +2135,7 @@
       <c r="AP2" s="39"/>
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A3" s="127"/>
+      <c r="A3" s="116"/>
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
@@ -2243,7 +2243,7 @@
       <c r="AP3" s="8"/>
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A4" s="127"/>
+      <c r="A4" s="116"/>
       <c r="B4" s="1" t="s">
         <v>42</v>
       </c>
@@ -2297,11 +2297,11 @@
       <c r="AP4" s="8"/>
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A5" s="127"/>
-      <c r="B5" s="119" t="s">
+      <c r="A5" s="116"/>
+      <c r="B5" s="118" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="119" t="s">
+      <c r="C5" s="118" t="s">
         <v>34</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -2347,9 +2347,9 @@
       <c r="AP5" s="8"/>
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A6" s="127"/>
-      <c r="B6" s="119"/>
-      <c r="C6" s="119"/>
+      <c r="A6" s="116"/>
+      <c r="B6" s="118"/>
+      <c r="C6" s="118"/>
       <c r="D6" s="3" t="s">
         <v>18</v>
       </c>
@@ -2455,7 +2455,7 @@
       <c r="AP6" s="8"/>
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A7" s="127"/>
+      <c r="A7" s="116"/>
       <c r="B7" s="3" t="s">
         <v>43</v>
       </c>
@@ -2510,7 +2510,7 @@
       <c r="AP7" s="8"/>
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A8" s="127"/>
+      <c r="A8" s="116"/>
       <c r="B8" s="3" t="s">
         <v>44</v>
       </c>
@@ -2566,7 +2566,7 @@
       <c r="AP8" s="10"/>
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A9" s="127"/>
+      <c r="A9" s="116"/>
       <c r="B9" s="3" t="s">
         <v>45</v>
       </c>
@@ -2622,7 +2622,7 @@
       <c r="AP9" s="10"/>
     </row>
     <row r="10" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A10" s="127"/>
+      <c r="A10" s="116"/>
       <c r="B10" s="3" t="s">
         <v>46</v>
       </c>
@@ -2678,7 +2678,7 @@
       <c r="AP10" s="10"/>
     </row>
     <row r="11" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A11" s="127"/>
+      <c r="A11" s="116"/>
       <c r="B11" s="3" t="s">
         <v>47</v>
       </c>
@@ -2734,11 +2734,11 @@
       <c r="AP11" s="10"/>
     </row>
     <row r="12" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A12" s="127"/>
-      <c r="B12" s="119" t="s">
+      <c r="A12" s="116"/>
+      <c r="B12" s="118" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="119" t="s">
+      <c r="C12" s="118" t="s">
         <v>22</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -2790,9 +2790,9 @@
       <c r="AP12" s="10"/>
     </row>
     <row r="13" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A13" s="127"/>
-      <c r="B13" s="119"/>
-      <c r="C13" s="119"/>
+      <c r="A13" s="116"/>
+      <c r="B13" s="118"/>
+      <c r="C13" s="118"/>
       <c r="D13" s="1" t="s">
         <v>24</v>
       </c>
@@ -2841,9 +2841,9 @@
       <c r="AP13" s="10"/>
     </row>
     <row r="14" spans="1:42" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="127"/>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
+      <c r="A14" s="116"/>
+      <c r="B14" s="118"/>
+      <c r="C14" s="118"/>
       <c r="D14" s="1" t="s">
         <v>18</v>
       </c>
@@ -2892,7 +2892,7 @@
       <c r="AP14" s="10"/>
     </row>
     <row r="15" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A15" s="127"/>
+      <c r="A15" s="116"/>
       <c r="B15" s="3" t="s">
         <v>39</v>
       </c>
@@ -2948,11 +2948,11 @@
       <c r="AP15" s="10"/>
     </row>
     <row r="16" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="A16" s="127"/>
-      <c r="B16" s="119" t="s">
+      <c r="A16" s="116"/>
+      <c r="B16" s="118" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="119" t="s">
+      <c r="C16" s="118" t="s">
         <v>20</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -3004,9 +3004,9 @@
       <c r="AP16" s="10"/>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A17" s="127"/>
-      <c r="B17" s="119"/>
-      <c r="C17" s="119"/>
+      <c r="A17" s="116"/>
+      <c r="B17" s="118"/>
+      <c r="C17" s="118"/>
       <c r="D17" s="1" t="s">
         <v>17</v>
       </c>
@@ -3055,9 +3055,9 @@
       <c r="AP17" s="10"/>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A18" s="127"/>
-      <c r="B18" s="119"/>
-      <c r="C18" s="119"/>
+      <c r="A18" s="116"/>
+      <c r="B18" s="118"/>
+      <c r="C18" s="118"/>
       <c r="D18" s="1" t="s">
         <v>18</v>
       </c>
@@ -3115,11 +3115,11 @@
       <c r="AP18" s="10"/>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A19" s="127"/>
-      <c r="B19" s="119" t="s">
+      <c r="A19" s="116"/>
+      <c r="B19" s="118" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="119" t="s">
+      <c r="C19" s="118" t="s">
         <v>36</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -3169,9 +3169,9 @@
       <c r="AP19" s="10"/>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A20" s="127"/>
-      <c r="B20" s="119"/>
-      <c r="C20" s="119"/>
+      <c r="A20" s="116"/>
+      <c r="B20" s="118"/>
+      <c r="C20" s="118"/>
       <c r="D20" s="1" t="s">
         <v>24</v>
       </c>
@@ -3215,9 +3215,9 @@
       <c r="AP20" s="10"/>
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A21" s="127"/>
-      <c r="B21" s="119"/>
-      <c r="C21" s="119"/>
+      <c r="A21" s="116"/>
+      <c r="B21" s="118"/>
+      <c r="C21" s="118"/>
       <c r="D21" s="1" t="s">
         <v>18</v>
       </c>
@@ -3296,7 +3296,7 @@
       <c r="AP21" s="10"/>
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A22" s="127"/>
+      <c r="A22" s="116"/>
       <c r="B22" s="3" t="s">
         <v>4</v>
       </c>
@@ -3351,7 +3351,7 @@
       <c r="AP22" s="10"/>
     </row>
     <row r="23" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A23" s="127"/>
+      <c r="A23" s="116"/>
       <c r="B23" s="3" t="s">
         <v>7</v>
       </c>
@@ -3406,7 +3406,7 @@
       <c r="AP23" s="10"/>
     </row>
     <row r="24" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A24" s="127"/>
+      <c r="A24" s="116"/>
       <c r="B24" s="3" t="s">
         <v>9</v>
       </c>
@@ -3463,7 +3463,7 @@
       <c r="AP24" s="10"/>
     </row>
     <row r="25" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A25" s="127"/>
+      <c r="A25" s="116"/>
       <c r="B25" s="3" t="s">
         <v>25</v>
       </c>
@@ -3518,7 +3518,7 @@
       <c r="AP25" s="10"/>
     </row>
     <row r="26" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A26" s="127"/>
+      <c r="A26" s="116"/>
       <c r="B26" s="3" t="s">
         <v>25</v>
       </c>
@@ -3573,11 +3573,11 @@
       <c r="AP26" s="10"/>
     </row>
     <row r="27" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A27" s="127"/>
-      <c r="B27" s="119" t="s">
+      <c r="A27" s="116"/>
+      <c r="B27" s="118" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="119" t="s">
+      <c r="C27" s="118" t="s">
         <v>27</v>
       </c>
       <c r="D27" s="3" t="s">
@@ -3628,9 +3628,9 @@
       <c r="AP27" s="10"/>
     </row>
     <row r="28" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A28" s="127"/>
-      <c r="B28" s="119"/>
-      <c r="C28" s="119"/>
+      <c r="A28" s="116"/>
+      <c r="B28" s="118"/>
+      <c r="C28" s="118"/>
       <c r="D28" s="3" t="s">
         <v>17</v>
       </c>
@@ -3679,7 +3679,7 @@
       <c r="AP28" s="10"/>
     </row>
     <row r="29" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A29" s="127"/>
+      <c r="A29" s="116"/>
       <c r="B29" s="3" t="s">
         <v>30</v>
       </c>
@@ -3736,7 +3736,7 @@
       <c r="AP29" s="10"/>
     </row>
     <row r="30" spans="1:43" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="127"/>
+      <c r="A30" s="116"/>
       <c r="B30" s="3" t="s">
         <v>37</v>
       </c>
@@ -3800,13 +3800,13 @@
       <c r="AP30" s="10"/>
     </row>
     <row r="31" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A31" s="133" t="s">
+      <c r="A31" s="115" t="s">
         <v>89</v>
       </c>
-      <c r="B31" s="117" t="s">
+      <c r="B31" s="134" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="117" t="s">
+      <c r="C31" s="134" t="s">
         <v>90</v>
       </c>
       <c r="D31" s="40" t="s">
@@ -3893,9 +3893,9 @@
       </c>
     </row>
     <row r="32" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A32" s="127"/>
-      <c r="B32" s="118"/>
-      <c r="C32" s="118"/>
+      <c r="A32" s="116"/>
+      <c r="B32" s="121"/>
+      <c r="C32" s="121"/>
       <c r="D32" s="1" t="s">
         <v>18</v>
       </c>
@@ -3955,7 +3955,7 @@
       </c>
     </row>
     <row r="33" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A33" s="127"/>
+      <c r="A33" s="116"/>
       <c r="B33" s="1" t="s">
         <v>68</v>
       </c>
@@ -4030,7 +4030,7 @@
       </c>
     </row>
     <row r="34" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A34" s="127"/>
+      <c r="A34" s="116"/>
       <c r="B34" s="1" t="s">
         <v>69</v>
       </c>
@@ -4114,7 +4114,7 @@
       </c>
     </row>
     <row r="35" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A35" s="127"/>
+      <c r="A35" s="116"/>
       <c r="B35" s="1" t="s">
         <v>70</v>
       </c>
@@ -4189,11 +4189,11 @@
       </c>
     </row>
     <row r="36" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A36" s="127"/>
-      <c r="B36" s="118" t="s">
+      <c r="A36" s="116"/>
+      <c r="B36" s="121" t="s">
         <v>71</v>
       </c>
-      <c r="C36" s="118" t="s">
+      <c r="C36" s="121" t="s">
         <v>97</v>
       </c>
       <c r="D36" s="1" t="s">
@@ -4273,9 +4273,9 @@
       </c>
     </row>
     <row r="37" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A37" s="127"/>
-      <c r="B37" s="118"/>
-      <c r="C37" s="118"/>
+      <c r="A37" s="116"/>
+      <c r="B37" s="121"/>
+      <c r="C37" s="121"/>
       <c r="D37" s="1" t="s">
         <v>29</v>
       </c>
@@ -4342,7 +4342,7 @@
       </c>
     </row>
     <row r="38" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A38" s="127"/>
+      <c r="A38" s="116"/>
       <c r="B38" s="1" t="s">
         <v>72</v>
       </c>
@@ -4433,7 +4433,7 @@
       </c>
     </row>
     <row r="39" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A39" s="127"/>
+      <c r="A39" s="116"/>
       <c r="B39" s="1" t="s">
         <v>73</v>
       </c>
@@ -4492,11 +4492,11 @@
       </c>
     </row>
     <row r="40" spans="1:43" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="127"/>
-      <c r="B40" s="120" t="s">
+      <c r="A40" s="116"/>
+      <c r="B40" s="133" t="s">
         <v>74</v>
       </c>
-      <c r="C40" s="119" t="s">
+      <c r="C40" s="118" t="s">
         <v>100</v>
       </c>
       <c r="D40" s="1" t="s">
@@ -4556,9 +4556,9 @@
       </c>
     </row>
     <row r="41" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A41" s="127"/>
-      <c r="B41" s="120"/>
-      <c r="C41" s="119"/>
+      <c r="A41" s="116"/>
+      <c r="B41" s="133"/>
+      <c r="C41" s="118"/>
       <c r="D41" s="1" t="s">
         <v>29</v>
       </c>
@@ -4638,7 +4638,7 @@
       </c>
     </row>
     <row r="42" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A42" s="127"/>
+      <c r="A42" s="116"/>
       <c r="B42" s="1" t="s">
         <v>75</v>
       </c>
@@ -4724,11 +4724,11 @@
       </c>
     </row>
     <row r="43" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A43" s="127"/>
-      <c r="B43" s="118" t="s">
+      <c r="A43" s="116"/>
+      <c r="B43" s="121" t="s">
         <v>76</v>
       </c>
-      <c r="C43" s="119" t="s">
+      <c r="C43" s="118" t="s">
         <v>121</v>
       </c>
       <c r="D43" s="1" t="s">
@@ -4786,9 +4786,9 @@
       </c>
     </row>
     <row r="44" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A44" s="127"/>
-      <c r="B44" s="118"/>
-      <c r="C44" s="119"/>
+      <c r="A44" s="116"/>
+      <c r="B44" s="121"/>
+      <c r="C44" s="118"/>
       <c r="D44" s="1" t="s">
         <v>94</v>
       </c>
@@ -4868,7 +4868,7 @@
       </c>
     </row>
     <row r="45" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A45" s="127"/>
+      <c r="A45" s="116"/>
       <c r="B45" s="1" t="s">
         <v>77</v>
       </c>
@@ -4959,11 +4959,11 @@
       </c>
     </row>
     <row r="46" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A46" s="127"/>
-      <c r="B46" s="118" t="s">
+      <c r="A46" s="116"/>
+      <c r="B46" s="121" t="s">
         <v>78</v>
       </c>
-      <c r="C46" s="119" t="s">
+      <c r="C46" s="118" t="s">
         <v>103</v>
       </c>
       <c r="D46" s="1" t="s">
@@ -5024,9 +5024,9 @@
       </c>
     </row>
     <row r="47" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A47" s="127"/>
-      <c r="B47" s="118"/>
-      <c r="C47" s="119"/>
+      <c r="A47" s="116"/>
+      <c r="B47" s="121"/>
+      <c r="C47" s="118"/>
       <c r="D47" s="1" t="s">
         <v>17</v>
       </c>
@@ -5106,7 +5106,7 @@
       </c>
     </row>
     <row r="48" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A48" s="127"/>
+      <c r="A48" s="116"/>
       <c r="B48" s="1" t="s">
         <v>79</v>
       </c>
@@ -5176,7 +5176,7 @@
       </c>
     </row>
     <row r="49" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A49" s="127"/>
+      <c r="A49" s="116"/>
       <c r="B49" s="1" t="s">
         <v>80</v>
       </c>
@@ -5246,7 +5246,7 @@
       </c>
     </row>
     <row r="50" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A50" s="127"/>
+      <c r="A50" s="116"/>
       <c r="B50" s="1" t="s">
         <v>81</v>
       </c>
@@ -5316,7 +5316,7 @@
       </c>
     </row>
     <row r="51" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A51" s="127"/>
+      <c r="A51" s="116"/>
       <c r="B51" s="1" t="s">
         <v>82</v>
       </c>
@@ -5386,7 +5386,7 @@
       </c>
     </row>
     <row r="52" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A52" s="127"/>
+      <c r="A52" s="116"/>
       <c r="B52" s="1" t="s">
         <v>83</v>
       </c>
@@ -5456,7 +5456,7 @@
       </c>
     </row>
     <row r="53" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A53" s="127"/>
+      <c r="A53" s="116"/>
       <c r="B53" s="1" t="s">
         <v>84</v>
       </c>
@@ -5526,7 +5526,7 @@
       </c>
     </row>
     <row r="54" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A54" s="127"/>
+      <c r="A54" s="116"/>
       <c r="B54" s="1" t="s">
         <v>85</v>
       </c>
@@ -5612,7 +5612,7 @@
       </c>
     </row>
     <row r="55" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A55" s="127"/>
+      <c r="A55" s="116"/>
       <c r="B55" s="1" t="s">
         <v>86</v>
       </c>
@@ -5698,7 +5698,7 @@
       </c>
     </row>
     <row r="56" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A56" s="127"/>
+      <c r="A56" s="116"/>
       <c r="B56" s="1" t="s">
         <v>87</v>
       </c>
@@ -5784,7 +5784,7 @@
       </c>
     </row>
     <row r="57" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A57" s="127"/>
+      <c r="A57" s="116"/>
       <c r="B57" s="1" t="s">
         <v>88</v>
       </c>
@@ -5870,7 +5870,7 @@
       </c>
     </row>
     <row r="58" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A58" s="127"/>
+      <c r="A58" s="116"/>
       <c r="B58" s="1" t="s">
         <v>117</v>
       </c>
@@ -5942,11 +5942,11 @@
       </c>
     </row>
     <row r="59" spans="1:43" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="127"/>
-      <c r="B59" s="118" t="s">
+      <c r="A59" s="116"/>
+      <c r="B59" s="121" t="s">
         <v>123</v>
       </c>
-      <c r="C59" s="118" t="s">
+      <c r="C59" s="121" t="s">
         <v>127</v>
       </c>
       <c r="D59" s="1" t="s">
@@ -6001,9 +6001,9 @@
       </c>
     </row>
     <row r="60" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A60" s="127"/>
-      <c r="B60" s="118"/>
-      <c r="C60" s="118"/>
+      <c r="A60" s="116"/>
+      <c r="B60" s="121"/>
+      <c r="C60" s="121"/>
       <c r="D60" s="1" t="s">
         <v>17</v>
       </c>
@@ -6061,11 +6061,11 @@
       </c>
     </row>
     <row r="61" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A61" s="127"/>
-      <c r="B61" s="118" t="s">
+      <c r="A61" s="116"/>
+      <c r="B61" s="121" t="s">
         <v>124</v>
       </c>
-      <c r="C61" s="119" t="s">
+      <c r="C61" s="118" t="s">
         <v>128</v>
       </c>
       <c r="D61" s="1" t="s">
@@ -6125,9 +6125,9 @@
       </c>
     </row>
     <row r="62" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A62" s="127"/>
-      <c r="B62" s="118"/>
-      <c r="C62" s="119"/>
+      <c r="A62" s="116"/>
+      <c r="B62" s="121"/>
+      <c r="C62" s="118"/>
       <c r="D62" s="1" t="s">
         <v>129</v>
       </c>
@@ -6185,11 +6185,11 @@
       </c>
     </row>
     <row r="63" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A63" s="127"/>
-      <c r="B63" s="118" t="s">
+      <c r="A63" s="116"/>
+      <c r="B63" s="121" t="s">
         <v>125</v>
       </c>
-      <c r="C63" s="119" t="s">
+      <c r="C63" s="118" t="s">
         <v>131</v>
       </c>
       <c r="D63" s="1" t="s">
@@ -6249,9 +6249,9 @@
       </c>
     </row>
     <row r="64" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A64" s="127"/>
-      <c r="B64" s="118"/>
-      <c r="C64" s="119"/>
+      <c r="A64" s="116"/>
+      <c r="B64" s="121"/>
+      <c r="C64" s="118"/>
       <c r="D64" s="1" t="s">
         <v>18</v>
       </c>
@@ -6309,7 +6309,7 @@
       </c>
     </row>
     <row r="65" spans="1:43" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="127"/>
+      <c r="A65" s="116"/>
       <c r="B65" s="1" t="s">
         <v>126</v>
       </c>
@@ -6378,7 +6378,7 @@
       </c>
     </row>
     <row r="66" spans="1:43" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="133" t="s">
+      <c r="A66" s="115" t="s">
         <v>140</v>
       </c>
       <c r="B66" s="40" t="s">
@@ -6444,11 +6444,11 @@
       <c r="AP66" s="39"/>
     </row>
     <row r="67" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A67" s="127"/>
-      <c r="B67" s="118" t="s">
+      <c r="A67" s="116"/>
+      <c r="B67" s="121" t="s">
         <v>152</v>
       </c>
-      <c r="C67" s="118" t="s">
+      <c r="C67" s="121" t="s">
         <v>153</v>
       </c>
       <c r="D67" s="1" t="s">
@@ -6505,9 +6505,9 @@
       <c r="AP67" s="8"/>
     </row>
     <row r="68" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A68" s="127"/>
-      <c r="B68" s="118"/>
-      <c r="C68" s="118"/>
+      <c r="A68" s="116"/>
+      <c r="B68" s="121"/>
+      <c r="C68" s="121"/>
       <c r="D68" s="1" t="s">
         <v>18</v>
       </c>
@@ -6562,11 +6562,11 @@
       <c r="AP68" s="8"/>
     </row>
     <row r="69" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A69" s="127"/>
-      <c r="B69" s="118" t="s">
+      <c r="A69" s="116"/>
+      <c r="B69" s="121" t="s">
         <v>154</v>
       </c>
-      <c r="C69" s="118" t="s">
+      <c r="C69" s="121" t="s">
         <v>155</v>
       </c>
       <c r="D69" s="1" t="s">
@@ -6623,9 +6623,9 @@
       <c r="AP69" s="8"/>
     </row>
     <row r="70" spans="1:43" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="134"/>
-      <c r="B70" s="118"/>
-      <c r="C70" s="118"/>
+      <c r="A70" s="117"/>
+      <c r="B70" s="121"/>
+      <c r="C70" s="121"/>
       <c r="D70" s="1" t="s">
         <v>29</v>
       </c>
@@ -6681,7 +6681,7 @@
       <c r="AP70" s="47"/>
     </row>
     <row r="71" spans="1:43" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="135" t="s">
+      <c r="A71" s="119" t="s">
         <v>141</v>
       </c>
       <c r="B71" s="40" t="s">
@@ -6744,7 +6744,7 @@
       <c r="AP71" s="8"/>
     </row>
     <row r="72" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A72" s="136"/>
+      <c r="A72" s="120"/>
       <c r="B72" s="1" t="s">
         <v>146</v>
       </c>
@@ -6805,7 +6805,7 @@
       <c r="AP72" s="8"/>
     </row>
     <row r="73" spans="1:43" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="136"/>
+      <c r="A73" s="120"/>
       <c r="B73" s="1" t="s">
         <v>148</v>
       </c>
@@ -6866,13 +6866,13 @@
       <c r="AP73" s="8"/>
     </row>
     <row r="74" spans="1:43" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="133" t="s">
+      <c r="A74" s="115" t="s">
         <v>143</v>
       </c>
-      <c r="B74" s="117" t="s">
+      <c r="B74" s="134" t="s">
         <v>157</v>
       </c>
-      <c r="C74" s="115" t="s">
+      <c r="C74" s="135" t="s">
         <v>165</v>
       </c>
       <c r="D74" s="40" t="s">
@@ -6930,9 +6930,9 @@
       <c r="AP74" s="39"/>
     </row>
     <row r="75" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A75" s="127"/>
-      <c r="B75" s="118"/>
-      <c r="C75" s="116"/>
+      <c r="A75" s="116"/>
+      <c r="B75" s="121"/>
+      <c r="C75" s="136"/>
       <c r="D75" s="1" t="s">
         <v>17</v>
       </c>
@@ -6987,7 +6987,7 @@
       <c r="AP75" s="8"/>
     </row>
     <row r="76" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A76" s="127"/>
+      <c r="A76" s="116"/>
       <c r="B76" s="3" t="s">
         <v>171</v>
       </c>
@@ -7050,7 +7050,7 @@
       </c>
     </row>
     <row r="77" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A77" s="127"/>
+      <c r="A77" s="116"/>
       <c r="B77" s="3" t="s">
         <v>172</v>
       </c>
@@ -7114,11 +7114,11 @@
       <c r="AP77" s="8"/>
     </row>
     <row r="78" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A78" s="127"/>
-      <c r="B78" s="119" t="s">
+      <c r="A78" s="116"/>
+      <c r="B78" s="118" t="s">
         <v>173</v>
       </c>
-      <c r="C78" s="119" t="s">
+      <c r="C78" s="118" t="s">
         <v>169</v>
       </c>
       <c r="D78" s="1" t="s">
@@ -7175,9 +7175,9 @@
       <c r="AP78" s="8"/>
     </row>
     <row r="79" spans="1:43" x14ac:dyDescent="0.2">
-      <c r="A79" s="127"/>
-      <c r="B79" s="119"/>
-      <c r="C79" s="119"/>
+      <c r="A79" s="116"/>
+      <c r="B79" s="118"/>
+      <c r="C79" s="118"/>
       <c r="D79" s="1" t="s">
         <v>94</v>
       </c>
@@ -7232,7 +7232,7 @@
       <c r="AP79" s="8"/>
     </row>
     <row r="80" spans="1:43" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="134"/>
+      <c r="A80" s="117"/>
       <c r="B80" s="99" t="s">
         <v>174</v>
       </c>
@@ -7335,6 +7335,35 @@
     </row>
   </sheetData>
   <mergeCells count="45">
+    <mergeCell ref="C74:C75"/>
+    <mergeCell ref="B74:B75"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="AJ1:AP1"/>
+    <mergeCell ref="X1:AC1"/>
+    <mergeCell ref="R1:W1"/>
+    <mergeCell ref="A2:A30"/>
+    <mergeCell ref="AD1:AI1"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="L1:Q1"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="A74:A80"/>
     <mergeCell ref="B12:B14"/>
     <mergeCell ref="C12:C14"/>
@@ -7351,35 +7380,6 @@
     <mergeCell ref="A31:A65"/>
     <mergeCell ref="B43:B44"/>
     <mergeCell ref="C43:C44"/>
-    <mergeCell ref="AJ1:AP1"/>
-    <mergeCell ref="X1:AC1"/>
-    <mergeCell ref="R1:W1"/>
-    <mergeCell ref="A2:A30"/>
-    <mergeCell ref="AD1:AI1"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="F1:K1"/>
-    <mergeCell ref="L1:Q1"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="C74:C75"/>
-    <mergeCell ref="B74:B75"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="C63:C64"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="E1:E1048576">

</xml_diff>